<commit_message>
chore: pin Streamlit Cloud to Python 3.10 for SciPy compatibility
</commit_message>
<xml_diff>
--- a/notebooks/Cleaned_Topic_Headlines.xlsx
+++ b/notebooks/Cleaned_Topic_Headlines.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1982,6 +1982,42 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>45894</v>
+      </c>
+      <c r="B44" t="n">
+        <v>6439.31982421875</v>
+      </c>
+      <c r="C44" t="n">
+        <v>6466.89013671875</v>
+      </c>
+      <c r="D44" t="n">
+        <v>6438.06005859375</v>
+      </c>
+      <c r="E44" t="n">
+        <v>6457.669921875</v>
+      </c>
+      <c r="F44" t="n">
+        <v>4059070000</v>
+      </c>
+      <c r="G44" t="n">
+        <v>-0.0042663855480634</v>
+      </c>
+      <c r="H44" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>inventhelp inventor develop new thermal capacitor water heater tl council asked to help expand eye on the street program gray medium to produce and air tomorrow new orleans saint preseason game in endtoend native hdr via nextgen tv hidden google search feature that make you a power user jerome powell signal fed may cut rate soon even a inflation risk remain elon musk must face lawsuit for duping trump supporter in million giveaway give your teeth the care they deserve with off an aquasonic ultra whitening toothbrush u supreme court allows nih to cut billion in research grant nature ninepoint partner announces estimated august cash distribution for ninepoint cash management fund etf series clean smarter not harder the best electric spin scrubber make cleaning a breeze federal workforce to lose employee this year trump official say in canada billboard woman in music open nomination for honoree cracker barrel crackup how the culture war are upending corporate branding powell signal fed may cut rate soon even a inflation risk remain canada will match u tariff exemption under usmca trade pact prime minister carney say whats needed to unlock the power and promise of imec new rv provides opioid recovery medical care to underserved minneapolis neighborhood powell signal fed may cut rate soon even a inflation risk remain onlyfans stats that show how massive the platform ha become green space are key to combating record heat in marginalized community familyfriendly workplace gov order budget cut for all state agency except school why xrp is soaring today are you even ready to grow lesson every owneroperator need before adding a truck gen z career catfishing rise ai recruiter a ethical solution trump say canada will drop usmcacompliant retaliatory tariff capital solution hire former caci exec a chief operating officer sunflower elect new board leader director king island tease return of beloved phantom theater ride top evercore analyst boost nvidia nvda stock price target ahead of q earnings tipranks bank lobby for national standard to limit state regulation shareholder alert levi korsinsky llp notifies investor it ha filed a complaint to recover loss suffered by purchaser of cai inc security and set a lead plaintiff deadline of october rosen national investor counsel encourages lockheed martin corporation investor to secure counsel before important deadline in security class action lmt elite express holding inc announces closing of million initial public offering ross benefit from value shopper but tariff challenge continue cvcc board set to review tax implication of new career center best ai writing tool for researcher zumpano patricios welcome sebastian jaramillo a income partner strengthening real estate practice zumpano patricios welcome sebastian jaramillo a income partner strengthening real estate practice canada to ease most retaliatory tariff against united state extrump cfo weisselberg may keep severance pay appellate court rule ethylene buyer could be ruined for their cartel example of unpaid work deal dispatch muskaltman drama ashton kutcher soho house play and we pose question to private equity pro fiserv push embedded payment for health care canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal netskope file for u ipo with m revenue yoy growth walmart q revenue surge to b raise fullyear outlook delta airline offering new direct flight from austin airport why intuit stock intu is sinking today blue bell ice cream recalled due to packaging error trump say hell be very good to canada a it prime minister drop some tariff trump say we want to be very good to canada a it leader drop some tariff canada remove some of it retaliatory tariff on the u canada remove some of it retaliatory tariff on the u canada remove some of it retaliatory tariff on the u npr trump say we want to be very good to canada a it leader drop some tariff canada remove some of it retaliatory tariff on the u weekly commodity wrapup why lucid group stock died today then got better tinley park chamber cancel this year oktoberfest due to cost how market reacted after powell signaled potential rate cut eastgroup property announces dividend increase how nvidias chip became central to the uschina trade war how nvidias chip became central to the uschina trade war how nvidias chip became central to the uschina trade war how nvidias chip became central to the uschina trade war branded legacy inc form strategic partnership with stanford university dr eran bendavid to advance addiction solution stock market surge after jerome powell indicates rate cut may be coming canada remove countertariffs on some u good canada to drop countertariffs on some u good one day after call with trump bitcoin and crypto stock surge a powell ratecut hint revives risk appetite walmart hike discount for shopper amid tariff uncertainty this is what whale are betting on okta starbucks car toy close on broadway in denver coffee giant closing all non drivethrus snap investor with loss in excess of k have opportunity to lead snap inc security lawsuit kirby mcinerney llp announces investigation against avita medical inc on behalf of investor bear alley marketing position itself a a leader in performance marketing for home service trump say hell keep extending tiktok shutdown deadline let talk indianola school business official brian bartz what is credit card forbearance and who qualifies for it this september bet bonus code nypbet bet get in bonus bet win or lose for yankee v red sox on friday sima monthly investment fund statistic july pi down from ath icp volume tank meanwhile blockdags b token sold point to the next x dsw offer discount on brook revel running shoe this week degree capital announces result of special meeting of shareholder to approve the proposed business combination with mount logan capital inc brattleboro parking zone to be relabeled high roller announces nyse acceptance of plan to regain listing compliance degree capital announces result of special meeting of shareholder to approve the proposed business combination with mount logan capital inc canada to remove many retaliatory tariff on u good allegro stock recovery elliott wave structure support fundamental case labubu blind box restocking aug aug here what to know trump say intel ha agreed to give the u a equity stake bloomberg rich lowry trump is wrong about mailin voting cheap drug high stake america risky bet on china trump again give putin a couple of week with no sign of ukraine peace talk underway cnn trump suggests chicago is next for federal crime crackdown followed by new york city cbs news president donald trump plan crime crackdown in chicago similar to dc national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital court ruling clear the way for hundred of cdc staff to be laid off jury selection taking time in randolph csc trial mayor trump president fixates on local crime asphalt and lamppost latest news on fbi searching john boltons home office george mason illegally used race in hiring department of education find george mason illegally used race in hiring department of education find a judge ha ordered alligator alcatraz in florida to wind down operation what happens now world cup draw will be held at washington kennedy center trump say kamala harris will take her day book tour to los angeles california gov gavin newsoms national profile soar with latest trump fight but there are risk california gov gavin newsoms national profile soar with latest trump fight but there are risk california gov gavin newsoms national profile soar with latest trump fight but there are risk newsoms profile soar with trump redistricting fight california gov gavin newsoms national profile soar with latest trump fight but there are risk california gov gavin newsoms national profile soar with latest trump fight but there are risk california gov gavin newsoms national profile soar with latest trump fight but there are risk lake lynn answer ferc question raise possibility of entry fee at cheat lake park people officially became u citizen at the new york state fair funeral home owner who stashed nearly decaying body set to be sentenced new york city to get federal police for crime crackdown after dc chicago trump trump praise missouri republican for considering redistricting bolton investigated over classified document not politics vp vance tell nbc community patrol confronts ice officer at city height elementary school parking lot stitt take aim at tulsa mayor decision to prosecute crime in tribal court trump tariff will reduce deficit by trillion over next decade say cbo report ask rusty how do i apply for s and receive my payment trump say hell keep extending tiktok shutdown deadline trump say hell keep extending tiktok shutdown deadline trump say hell keep extending tiktok shutdown deadline trump say hell keep extending tiktok shutdown deadline uk diplomat receives warning over illegal fishing with jd vance mit global collapse warning revisited humanity enters makeorbreak decade chicago is up next for the national guard theyre screaming for u say trump san carlos and the lastminute commissioner item henderson accepting application for addition to veteran memorial wall trump reacts to canada reversing retaliatory tariff take question at white house erik and lyle menendez can still walk free from prison even if both brother have parole denied a family fight back desantis fire back after dem decries florida move to ditch lgbt rainbow color from crosswalk in orlando hegseth authorizes national guard to carry gun in washington dc ap technology summarybrief at pm edt trump is astonishingly deluded about putin trump official demand apology from george mason president over diversity the new york time the u air force just underwent a massive stress test of how it would fight a highend war in the pacific uk top diplomat get a warning for illegal fishing with u vice president national guard troop in washington will be armed hegseth matt fleming how assembly democrat came to embrace gerrymandering passing the baton in europe could donald trump really win the nobel peace prize asking eric am i wrong for wanting to back out of mexican vacation now that friend included her son beware of the skeeters and malary asking eric am i wrong for backing out of a trip because a friend son is going an energy transition at the crossroad south korea journey toward resilience the u navy drone effort arent going wellbut neither are china pa budget stall again what will it take to break the cycle of delay carney say he will travel to germany next week to deepen tie canada go learn some english customer berates georgian nyc cafe owner now everyones coming to her defense teaching just the fact is not an answer to indoctrination gavin newsoms redistricting gambit a presidential audition not a policy plan fifa world cup draw to take place at kennedy center trump announces tension flare a texas house panel hears a bathroom bill for first time in eight year trump message to dc criminal democrat dont mess with me how some apps are working to solve the epidemic of loneliness what to expect from the ussouth korea summit planned parenthood sue south carolina over medicaid ban certain local voice oppose gov newsoms redistricting campaign cracker barrel new logo sucksand not because of wokeness you idiot ct governor directs flag to halfstaff saturday for state employee fatally injured on job trump say hell ask congress for b for dc improvement letter taxpayer against genocide trump say putin may attend north america world cup it so on after heated back and forth with chris rufo on conservatism jonah goldberg agrees to debate homeowner oppose plan for fencing dune on hollywood beach here why trump say putin may attend north america world cup california ab stall in senate amid parental right opposition trump say putin may attend north america world cup trump say putin may attend north america world cup california governor signed a redistricting plan what happens next trump show off photo putin mailed him from alaska summit but president warns i better be very happy with peace talk after russia ukraine attack policy review committee recap august james jim mcgregor trump say chicago is next for dcstyle federal law enforcement operation a judge ha ordered alligator alcatraz in florida to wind down operation what happens now a judge ha ordered alligator alcatraz in florida to wind down operation what happens now a judge ha ordered alligator alcatraz in florida to wind down operation what happens now a judge ha ordered alligator alcatraz in florida to wind down operation what happens now a judge ha ordered alligator alcatraz in florida to wind down operation what happens now a judge ha ordered alligator alcatraz in florida to wind down operation what happens now shiba inu shib is taking longer than expected to reach new high in pepe coin pepe and this coin to outperform it investing in ozak ai ethereumbased ai token during it under presale could lead to millionaire status by a btc and eth hit ath cadence bank ha million stock holding in texas instrument incorporated txn jpmorgan chase co jpm share sold by rbo co llc hoka ha shoe on sale for a low a right now including bondi and clifton trump administration halt construction of revolution wind farm off mass citing national security new brewery tap into corydons dora ordinance excitement british columbia investment management corp sell share of alphabet inc goog british columbia investment management corp raise holding in broadcom inc avgo air canada say more passenger eligible for reimbursement if flight were cancelled canada grab these safe djia dividend bargain after index hit alltime high nextgen pick best cryptos to buy today a arctic pablos cex listing driving maximum gain potential twothirds of river trash is plastic research fastfood chain lock in meal to fight inflation in newsguild see organizing surge a medium worker fuel grassroots militancy tech ceo urge dignity for billion shift worker amid automation lowes target pro with total home strategy amid sale dip and inflation european postal service halt u shipment over trump tariff china stock surge defies weak economy raising fear of another bust analyst waste management inc nysewm announces quarterly dividend evans city council approves ballot language for permanent road tax bet bonus code orl bonus for seahawks v packer raider v cardinal solana whale rotate capital into layer brett analyst say it could deliver x gain by next year whale are choosing this meme coin a the best crypto to buy in instead of dogecoin doge and shiba sol strengthens on institutional demand xrp jump after whale action and blockdags forecast draw buyer in phoenix wealth advisor sell share of air product and chemical inc apd btc climbed to of global money before fed chair signaled rate cut cointelegraph heritage wealth partner llc buy share of meta platform inc meta palantir technology nasdaqpltr insider ryan taylor sell share palantir technology nasdaqpltr insider ryan taylor sell share of stock promising retail stock to keep an eye on august th jpmorgan chase co jpm is biondo investment advisor llcs th largest position immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say trump appeal in fraud case likely despite his total victory trump appeal in fraud case likely despite his total victory baby boomer turned meme stock trading into a thrilling hobby calling it absolutely gambling trump appeal in fraud case likely despite his total victory this weatherproof storage shed is only during wayfairs labor day blowout sale bank of america nysebac hit new month high whats next invesco qqq qqq share purchased by haverford trust co cardano price prediction ada eye new high yet this lowcap coin ha x more upside beltway buzz august apg asset management nv acquires share of intuitive surgical inc isrg pfizer inc pfe share sold by apg asset management nv what to know about visa for foreign trucker and the politics of a deadly florida crash the best amazon deal to shop right now save up to trump halt work on new england offshore wind project thats nearly complete trump halt work on new england offshore wind project thats nearly complete bitcoin btc price could retrace before a run toward kk but ripple xrp and this coin are aiming high in cryptos next top altcoin why this crypto could shine a xrp fall below best gift for digital artist in trump halt work on nearly complete new england offshore wind project waste management inc wm share acquired by groupe la francaise union pacific corporation unp share purchased by kestra advisory service llc haverford trust co sell share of unitedhealth group incorporated unh waste management inc wm share sold by van hulzen asset management llc groupe la francaise purchase share of walmart inc wmt phoenix wealth advisor trim position in cisco system inc csco bahl gaynor inc increase stake in taiwan semiconductor manufacturing company ltd tsm best of the best bahl gaynor inc sell share of mcdonalds corporation mcd chicago a mess trump vow national guard crackdown layer brett dubbed pepe after early momentum outpaces early doge and shib launch hooter bankruptcy prompt rebrand to tacky familyfriendly are home depot cheapest tool set worth buying here what user say trump halt work on new england offshore wind project thats nearly complete douglas winthrop advisor llc sell share of pepsico inc pep caitlin john llc ha holding in invesco qqq qqq british columbia investment management corp buy share of procter gamble company the pg penticton council willing to work with art gallery after layoff announced penticton get your own steam locomotive how family can save money this backtoschool season northwest minnesota foundation issue over million in grant loan during th quarter why the iea reinstated it business a usual scenario business accelerator academy start in september how u of a help build worldclass entrepreneur dogecoin price target in september but analyst say x gain belong to new lowcaps can solana reach by or is there a better crypto to buy now blockdags m presale and referral reward shift focus from xrp rally and eth market issue trump halt work on new england offshore wind project thats nearly complete yahoocom trump halt work on new england offshore wind project thats nearly complete trump halt work on new england offshore wind project thats nearly complete ai bubble fear spark tech stock slide crash warning rise how and where to bet mlb player prop pick odds for aug garrett crochet among best bet smartleaf asset management llc ha million stock holding in mastercard incorporated ma walmart nysewmt issue fy earnings guidance biondo investment advisor llc ha million stake in unitedhealth group incorporated unh cadence bank sell share of american express company axp forest avenue capital management lp boost holding in vistra corp vst european post suspend u delivery over trumpera tariff biondo investment advisor llc acquires share of amgen inc amgn svb wealth llc lower stock position in blackrock blk svb wealth llc sell share of air product and chemical inc apd air product and chemical inc apd share sold by british columbia investment management corp svb wealth llc sell share of air product and chemical inc apd lionshead wealth management llc ha holding in illinois tool work inc itw biondo investment advisor llc increase stock holding in duke energy corporation duk kruse out a dia director in latest pentagon shakeup cringe watch zohran mamdani plan nyc scavenger hunt is there a prize if youre mugged on the subway cu colorado spring campus thought it could avoid trump education crackdown here what happened cu colorado spring campus thought it could avoid trump education crackdown here what happened cu colorado spring campus thought it could avoid trump education crackdown here what happened u justice department release transcript of interview with ghislaine maxwell kilmar abrego garcia is freed from tennessee jail so he can rejoin family in maryland to await trial greene issue scathing rebuke of condition in gaza i will not be silent about it israel vow to open gate of hell on gaza in chilling warning a famine grip the region u seek to deport kilmar abrego garcia to uganda after he refused plea offer in his smuggling case u seek to deport kilmar abrego garcia to uganda after he refused plea offer in his smuggling case kevin oleary sound alarm on rich kid upbringing they become lost in a sea of mediocrity it a disaster for them former dhs official signal he could be next after bolton fbi raid we expect it the lioness at the center of a city hall battered by scandal dnc vote on israel arm embargo may set democratic party course on palestine trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it u seek to deport abrego garcia to uganda hampton county law enforcement to ramp up duo patrol trump administration considering deporting kilmar abrego garcia to uganda his lawyer say secretariat jockey mourned in maine a well a canada dunkin customer warns to check receipt after spotting wellness fee national guard roll out in state not linked to trump crime crackdown wh say the redistricting war between texas and california is about to jolt the midterm politico asking eric were no longer invited to shared family holiday meal what should we do about upcoming wedding redistricting war poised to explode a california and texas make their move la consequential karen bass earns epic ratio over claim city recovery is fastest in state history the redistricting war between texas and california is about to jolt the midterm texas abbott promise quick signature of redistricting plan following overnight senate vote ghislaine maxwell absolves trump and everyone else in doj interview conservative activist slam cracker barrel a company left reeling after logo redesign south korea japan agree to boost tie a challenge mount kilmar abrego garcia released from ice custody after return from el salvador truck driver in crash at center of trump administration feud with newsom is denied bond when trying to explain low dem party polling look no further than awesome duo of newsom and swalwell immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say u seek to deport kilmar abrego garcia to uganda after he refused plea offer in his smuggling case trump look to chicago next in federal crackdown the wall street journal giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell university of oregon concludes law review discriminated based on perceived national origin against israeli author trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress how redistricting is done and why it could give party an edge in election how redistricting is done and why it could give party an edge in election democrat mock jd vance for having cardboard charisma a he push unpopular budget bill opinion it time for mayo pete buttigieg to find some seasoning what happened to ambition for bay restoration guest commentary kilmar abrego garcia threatened with deportation to uganda larimer county restaurant inspection made aug kilmar abrego garcia threatened with deportation to uganda kilmar abrego garcia threatened with deportation to uganda judge block trump from cutting funding from city and county including denver over sanctuary policy internet tax freedom act preempt new york imposition of tax fbi target john boltons home and office trump he not a smart guy but he could be a very unpatriotic guy inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal rachel bitecofer warns that bolton is just the start and trump will go after the rest of u inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal what we know about china and russia new strategic bomber inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal zelenskyy say security guarantee for ukraine to be ready soon bill maher applauds gavin newsom for mocking donald trump i think it very funny floridarun alligator alcatraz violates u law aclu say russia announces support for venezuela to defend sovereignty amid growing military tension with the united state gianno caldwell mull senate bid a chicagoans are begging for change on crime woe trump threatens chicago with next national guard invasion cnn analyst pinpoint the weirdest part of ghislaine maxwell simply bizarre doj interview cnn analyst pinpoint the weirdest part of ghislaine maxwell simply bizarre doj interview the owl eye liberty and memory from epstein suicide to trump and clinton takeaway from ghislaine maxwell transcript how can israel engineer a famine in gaza in the st century what we learned from the ghislaine maxwell doj interview texas gov abbott say hell swiftly sign redistricting map after lawmaker approve them jeff bezos said he would have felt icky had he taken any more share of amazon i just didnt feel good smart money strategy what the pro buy when the crypto market crash radioactive shrimp update walmart store brand and other brand recalled european postal service suspend shipment of package to u over tariff european postal service suspend shipment of package to u over tariff european postal service suspend shipment of package to u over tariff european postal service suspend shipment of package to u over tariff european postal service suspend shipment of package to u over tariff european postal service suspend shipment of package to u over tariff a winning powerball ticket ha been sold in western new york the sp hasnt yielded this little since the dotcom bubble here what investor can do the motley fool just ranked the biggest financial stock here why the no pick could be your best investment mezcal producer preserve traditional method a demand for liquor grows minute european postal service suspend shipment of package to u over tariff kpop demon hunter give netflix it first boxoffice win curry join the bank holiday sale bonanza with it epic deal event here are the best offer id buy self driving taxi may be coming to nyc a waymo win first av testing permit mashable rosen a leading law firm encourages fiserv inc investor to secure counsel before important rosen a leading law firm encourages fiserv inc investor to secure counsel before important rosen a leading law firm encourages fiserv inc investor to secure counsel before important rosen a leading law firm encourages fiserv inc investor to secure counsel before important rosen a leading law firm encourages fiserv inc investor to secure counsel before important deadline in security class action fi ice cream sold at walmarts across state recalled due to undeclared allergen here how a gamestop purchase turned into a bitcoin jackpot ice cream sold at walmarts across state recalled due to undeclared allergen fox business prediction lucid group sale will soar over the next year if this happens solar executive warn that trump attack on renewables will lead to power crunch that spike electricity price pueblo county home listing asked for less money in july see the current median price here prediction these trilliondollar artificial intelligence ai stock could strike a megadeal that wall street isnt ready for cold wallet cashback utility and presale pricing create a upside case while chainlink and shiba inu struggle maintenance compliance burden viability of hopi water treatment system ethereum in trouble xrp might breakout buyer turn to blockdag to earn referral reward acting a the executor of a will can be a very lucrative job the last word national guard troop to be force multiplier for ice homan little pepe crypto price prediction is lilpepe a good investment for longterm holder here how much you should aim to invest in the invesco qqq etf to get to million or more by retirement state audit question m in federal spending by moses lake school district blockchain stock worth watching august th owner scale back golden mile shopping center redevelopment rosen global investor counsel encourages easterly rocmuni high income municipal bond fund comerica bank lower stake in alphabet inc goog trump tap airbnb cofounder a st government design head to lead huge web overhaul trump tap airbnb cofounder a st government design head to lead huge web overhaul fox business offgrid living next new real estate trend a application for rural mortgage skyrocket rosen global investor counsel encourages altimmune inc investor to secure counsel before rosen global investor counsel encourages altimmune inc investor to secure counsel before rosen global investor counsel encourages altimmune inc investor to secure counsel before epstein accuser virginia giuffre wrote a memoir month after her death it coming out powell warning signal unemployment claim jump to highest in year cardano price outlook can ada reach trumprelated defi platform world liberty financial debut wlfi token on ethereum mainnet rosen global investor counsel encourages altimmune inc investor to secure counsel before important deadline in security class action alt the best meme coin presale stampede is loading whitelist labubull now or watch it moon without you backtoschool deal tellos unlimited plan get you cell service for per month your first month nexus gold cvenxs stock price up whats next mason resource cvellg stock price up here why mason resource cvellg trading up here what happened national guard troop to be force multiplier for ice homan freedom investment management inc purchase share of procter gamble company the pg ascent group llc raise stock holding in ameri</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>inventhelp inventor develop new thermal capacitor water heater tl council help expand eye street program gray medium produce air tomorrow new orleans saint preseason game endtoend native hdr via nextgen tv hidden google search feature power user jerome powell signal fed cut rate soon inflation risk elon musk must face lawsuit duping trump supporter million giveaway give teeth care deserve aquasonic ultra whitening toothbrush supreme court allows nih cut billion research grant nature ninepoint partner announces estimated august cash distribution ninepoint cash management fund etf series clean smarter harder best electric spin scrubber cleaning breeze federal workforce lose employee year trump canada billboard woman music open nomination honoree cracker barrel crackup culture war upending corporate branding powell signal fed cut rate soon inflation risk canada match tariff exemption usmca trade pact prime minister carney whats needed unlock power promise imec new rv provides opioid recovery medical care underserved minneapolis neighborhood powell signal fed cut rate soon inflation risk onlyfans stats massive platform become green space combating record heat marginalized community familyfriendly workplace gov order budget cut agency except school xrp soaring today ready grow lesson owneroperator adding truck gen z career catfishing rise ai recruiter ethical solution trump canada drop usmcacompliant retaliatory tariff capital solution hire caci exec chief operating officer sunflower elect new board director king island tease beloved phantom theater ride evercore analyst boost nvidia nvda stock price target ahead q earnings tipranks bank lobby national limit regulation shareholder alert levi korsinsky llp notifies investor filed complaint recover loss suffered purchaser cai security set lead plaintiff deadline october rosen national investor counsel encourages lockheed martin corporation investor secure counsel important deadline security class action lmt elite express holding announces closing million initial public offering ross benefit value shopper tariff challenge continue cvcc board set review tax implication new career center best ai writing tool researcher zumpano patricios welcome sebastian jaramillo income partner strengthening real estate practice zumpano patricios welcome sebastian jaramillo income partner strengthening real estate practice canada ease retaliatory tariff united extrump cfo weisselberg severance pay appellate court rule ethylene buyer ruined cartel example unpaid work deal dispatch muskaltman drama ashton kutcher soho house play pose private equity pro fiserv push embedded payment health care canada removing tariff good compliant free trade deal canada removing tariff good compliant free trade deal canada removing tariff good compliant free trade deal canada removing tariff good compliant free trade deal canada removing tariff good compliant free trade deal canada removing tariff good compliant free trade deal canada removing tariff good compliant free trade deal canada removing tariff good compliant free trade deal netskope file ipo revenue yoy growth walmart q revenue surge b raise fullyear outlook delta airline offering new direct flight austin airport intuit stock intu sinking today blue bell cream recalled due packaging error trump hell good canada prime minister drop tariff trump good canada drop tariff canada remove retaliatory tariff canada remove retaliatory tariff canada remove retaliatory tariff npr trump good canada drop tariff canada remove retaliatory tariff weekly commodity wrapup lucid stock died today got better tinley park chamber cancel year oktoberfest due cost market reacted powell signaled potential rate cut eastgroup property announces dividend increase nvidias chip became central uschina trade war nvidias chip became central uschina trade war nvidias chip became central uschina trade war nvidias chip became central uschina trade war branded legacy form strategic partnership stanford university dr eran bendavid advance addiction solution stock market surge jerome powell indicates rate cut coming canada remove countertariffs good canada drop countertariffs good day call trump bitcoin crypto stock surge powell ratecut hint revives risk appetite walmart hike discount shopper amid tariff uncertainty whale betting okta starbucks car toy close broadway denver coffee giant closing non drivethrus snap investor loss excess k opportunity lead snap security lawsuit kirby mcinerney llp announces investigation avita medical behalf investor bear alley marketing performance marketing service trump hell extending tiktok shutdown deadline indianola school business brian bartz credit card forbearance qualifies september bet bonus code nypbet bet bonus bet lose yankee v red sox friday sima monthly investment fund statistic july pi ath icp volume tank meanwhile blockdags b token sold next x dsw offer discount brook revel running shoe degree capital announces special meeting shareholder approve proposed business combination mount logan capital brattleboro parking zone relabeled high roller announces nyse acceptance plan regain listing compliance degree capital announces special meeting shareholder approve proposed business combination mount logan capital canada remove retaliatory tariff good allegro stock recovery elliott wave structure support fundamental case labubu blind box restocking aug aug trump intel agreed give equity stake bloomberg rich lowry trump mailin voting cheap drug high stake america risky bet china trump give putin couple sign ukraine peace underway cnn trump suggests chicago next federal crime crackdown followed new york cbs news president donald trump plan crime crackdown chicago similar dc national guard troop soon carry weapon capital national guard troop soon carry weapon capital national guard troop soon carry weapon capital national guard troop soon carry weapon capital national guard troop soon carry weapon capital national guard troop soon carry weapon capital national guard troop soon carry weapon capital national guard troop soon carry weapon capital court ruling cdc staff laid jury selection taking randolph csc trial mayor trump president fixates local crime asphalt lamppost latest news fbi searching john boltons office george mason illegally used race hiring department education find george mason illegally used race hiring department education find judge ordered alligator alcatraz florida wind operation happens world cup draw washington kennedy center trump kamala harris take day book tour los angeles california gov gavin newsoms national profile soar latest trump fight risk california gov gavin newsoms national profile soar latest trump fight risk california gov gavin newsoms national profile soar latest trump fight risk newsoms profile soar trump redistricting fight california gov gavin newsoms national profile soar latest trump fight risk california gov gavin newsoms national profile soar latest trump fight risk california gov gavin newsoms national profile soar latest trump fight risk lake lynn answer ferc raise possibility entry fee cheat lake park people officially became citizen new york fair funeral owner stashed nearly decaying body set sentenced new york federal police crime crackdown dc chicago trump trump praise missouri republican considering redistricting bolton investigated classified document politics vp vance nbc community patrol confronts officer height elementary school parking lot stitt take aim tulsa mayor decision prosecute crime tribal court trump tariff reduce deficit trillion next decade cbo report rusty apply receive payment trump hell extending tiktok shutdown deadline trump hell extending tiktok shutdown deadline trump hell extending tiktok shutdown deadline trump hell extending tiktok shutdown deadline uk diplomat receives warning illegal fishing jd vance mit global collapse warning revisited humanity enters makeorbreak decade chicago next national guard theyre screaming trump san carlos lastminute commissioner item henderson accepting application addition veteran memorial wall trump reacts canada reversing retaliatory tariff take white house erik lyle menendez walk free prison brother parole denied family fight desantis fire dem decries florida move ditch lgbt rainbow color crosswalk orlando hegseth authorizes national guard carry gun washington dc technology summarybrief pm trump astonishingly deluded putin trump demand apology george mason president diversity new york air force underwent massive stress test fight highend war pacific uk diplomat warning illegal fishing vice president national guard troop washington armed hegseth matt fleming assembly democrat came embrace gerrymandering passing baton europe donald trump nobel peace prize asking eric wanting mexican vacation friend included son beware skeeters malary asking eric backing trip friend son energy transition crossroad south korea journey resilience navy drone effort arent wellbut neither china pa budget stall take break cycle delay carney travel germany next deepen tie canada learn english customer berates georgian nyc cafe owner everyones coming defense teaching fact answer indoctrination gavin newsoms redistricting gambit presidential audition policy plan fifa world cup draw take place kennedy center trump announces tension flare texas house panel hears bathroom bill year trump message dc criminal democrat dont mess apps working solve epidemic loneliness expect ussouth korea summit planned parenthood sue south carolina medicaid ban certain local voice oppose gov newsoms redistricting campaign cracker barrel new logo sucksand wokeness idiot ct governor directs flag halfstaff saturday employee fatally injured job trump hell congress b dc improvement letter taxpayer genocide trump putin attend north america world cup heated forth chris rufo conservatism jonah goldberg agrees debate homeowner oppose plan fencing dune hollywood beach trump putin attend north america world cup california ab stall senate amid parental opposition trump putin attend north america world cup trump putin attend north america world cup california governor signed redistricting plan happens next trump photo putin mailed alaska summit president warns better happy peace russia ukraine attack policy review committee recap august james jim mcgregor trump chicago next dcstyle federal law enforcement operation judge ordered alligator alcatraz florida wind operation happens judge ordered alligator alcatraz florida wind operation happens judge ordered alligator alcatraz florida wind operation happens judge ordered alligator alcatraz florida wind operation happens judge ordered alligator alcatraz florida wind operation happens judge ordered alligator alcatraz florida wind operation happens shiba inu shib taking longer expected reach new high pepe coin pepe coin outperform investing ozak ai ethereumbased ai token presale lead millionaire status btc eth hit ath cadence bank million stock holding texas instrument incorporated txn jpmorgan chase co jpm share sold rbo co llc hoka shoe sale low bondi clifton trump administration halt construction revolution wind mass citing national security new brewery tap corydons dora ordinance excitement british columbia investment management corp sell share alphabet goog british columbia investment management corp raise holding broadcom avgo air canada passenger eligible reimbursement flight cancelled canada grab safe djia dividend bargain index hit alltime high nextgen pick best cryptos buy today arctic pablos cex listing driving maximum gain potential twothirds river trash plastic research fastfood chain lock meal fight inflation newsguild organizing surge medium worker fuel grassroots militancy tech ceo urge dignity billion shift worker amid automation lowes target pro total strategy amid sale dip inflation european postal service halt shipment trump tariff china stock surge defies weak economy raising fear another bust analyst waste management nysewm announces quarterly dividend evans council approves ballot language permanent road tax bet bonus code orl bonus seahawks v packer raider v cardinal solana whale rotate capital layer brett analyst deliver x gain next year whale choosing meme coin best crypto buy instead dogecoin doge shiba sol strengthens institutional demand xrp jump whale action blockdags forecast draw buyer phoenix wealth advisor sell share air product chemical apd btc climbed global money fed chair signaled rate cut cointelegraph heritage wealth partner llc buy share meta platform meta palantir technology nasdaqpltr insider ryan taylor sell share palantir technology nasdaqpltr insider ryan taylor sell share stock promising retail stock eye august jpmorgan chase co jpm biondo investment advisor llcs largest immigration boosted europe economy pandemic ecbs lagarde immigration boosted europe economy pandemic ecbs lagarde immigration boosted europe economy pandemic ecbs lagarde trump appeal fraud case likely total victory trump appeal fraud case likely total victory baby boomer turned meme stock trading thrilling hobby calling absolutely gambling trump appeal fraud case likely total victory weatherproof storage shed wayfairs labor day blowout sale bank america nysebac hit new month high whats next invesco qqq qqq share purchased haverford trust co cardano price prediction ada eye new high yet lowcap coin x upside beltway buzz august apg asset management nv acquires share intuitive surgical isrg pfizer pfe share sold apg asset management nv visa foreign trucker politics deadly florida crash best amazon deal shop save trump halt work new england offshore wind project thats nearly complete trump halt work new england offshore wind project thats nearly complete bitcoin btc price retrace run kk ripple xrp coin aiming high cryptos next altcoin crypto shine xrp fall best gift digital artist trump halt work nearly complete new england offshore wind project waste management wm share acquired groupe la francaise union pacific corporation unp share purchased kestra advisory service llc haverford trust co sell share unitedhealth incorporated unh waste management wm share sold van hulzen asset management llc groupe la francaise purchase share walmart wmt phoenix wealth advisor trim cisco system csco bahl gaynor increase stake taiwan semiconductor manufacturing company tsm best best bahl gaynor sell share mcdonalds corporation mcd chicago mess trump vow national guard crackdown layer brett dubbed pepe early momentum outpaces early doge shib launch hooter bankruptcy prompt rebrand tacky familyfriendly depot cheapest tool set worth buying user trump halt work new england offshore wind project thats nearly complete douglas winthrop advisor llc sell share pepsico pep caitlin john llc holding invesco qqq qqq british columbia investment management corp buy share procter gamble company pg penticton council willing work art gallery layoff announced penticton steam locomotive family save money backtoschool season northwest minnesota foundation issue million grant loan quarter iea reinstated business usual scenario business accelerator academy start september help build worldclass entrepreneur dogecoin price target september analyst x gain belong new lowcaps solana reach better crypto buy blockdags presale referral reward shift focus xrp rally eth market issue trump halt work new england offshore wind project thats nearly complete yahoocom trump halt work new england offshore wind project thats nearly complete trump halt work new england offshore wind project thats nearly complete ai bubble fear spark tech stock slide crash warning rise bet mlb player prop pick odds aug garrett crochet among best bet smartleaf asset management llc million stock holding mastercard incorporated walmart nysewmt issue fy earnings guidance biondo investment advisor llc million stake unitedhealth incorporated unh cadence bank sell share american express company axp forest avenue capital management lp boost holding vistra corp vst european post suspend delivery trumpera tariff biondo investment advisor llc acquires share amgen amgn svb wealth llc lower stock blackrock blk svb wealth llc sell share air product chemical apd air product chemical apd share sold british columbia investment management corp svb wealth llc sell share air product chemical apd lionshead wealth management llc holding illinois tool work itw biondo investment advisor llc increase stock holding duke energy corporation duk kruse dia director latest pentagon shakeup cringe watch zohran mamdani plan nyc scavenger hunt prize youre mugged subway cu colorado spring campus thought avoid trump education crackdown happened cu colorado spring campus thought avoid trump education crackdown happened cu colorado spring campus thought avoid trump education crackdown happened justice department release transcript interview ghislaine maxwell kilmar abrego garcia freed tennessee jail rejoin family maryland await trial greene issue scathing rebuke condition gaza silent israel vow open gate hell gaza chilling warning famine grip region seek deport kilmar abrego garcia uganda refused plea offer smuggling case seek deport kilmar abrego garcia uganda refused plea offer smuggling case kevin oleary sound alarm rich kid upbringing become sea mediocrity disaster dhs signal next bolton fbi raid expect lioness center hall battered scandal dnc vote israel arm embargo set democratic party course palestine trump ran promise revenge making good trump ran promise revenge making good trump ran promise revenge making good trump ran promise revenge making good trump ran promise revenge making good trump ran promise revenge making good trump ran promise revenge making good seek deport abrego garcia uganda hampton county law enforcement ramp duo patrol trump administration considering deporting kilmar abrego garcia uganda lawyer secretariat jockey mourned maine canada dunkin customer warns receipt spotting wellness fee national guard roll linked trump crime crackdown wh redistricting war texas california jolt midterm politico asking eric longer invited shared family holiday meal upcoming wedding redistricting war poised explode california texas move la consequential karen bass earns epic ratio claim recovery fastest history redistricting war texas california jolt midterm texas abbott promise quick signature redistricting plan following overnight senate vote ghislaine maxwell absolves trump everyone else doj interview conservative activist slam cracker barrel company left reeling logo redesign south korea japan agree boost tie challenge mount kilmar abrego garcia released custody el salvador truck driver crash center trump administration feud newsom denied bond explain low dem party polling look awesome duo newsom swalwell immigration boosted europe economy pandemic ecbs lagarde immigration boosted europe economy pandemic ecbs lagarde immigration boosted europe economy pandemic ecbs lagarde immigration boosted europe economy pandemic ecbs lagarde immigration boosted europe economy pandemic ecbs lagarde seek deport kilmar abrego garcia uganda refused plea offer smuggling case trump look chicago next federal crackdown wall street journal giuffre family outraged doj interview ghislaine maxwell giuffre family outraged doj interview ghislaine maxwell giuffre family outraged doj interview ghislaine maxwell giuffre family outraged doj interview ghislaine maxwell giuffre family outraged doj interview ghislaine maxwell giuffre family outraged doj interview ghislaine maxwell giuffre family outraged doj interview ghislaine maxwell university oregon concludes law review discriminated perceived national origin israeli author trump hail new texas electoral map aimed keeping grip congress trump hail new texas electoral map aimed keeping grip congress trump hail new texas electoral map aimed keeping grip congress trump hail new texas electoral map aimed keeping grip congress trump hail new texas electoral map aimed keeping grip congress trump hail new texas electoral map aimed keeping grip congress trump hail new texas electoral map aimed keeping grip congress trump hail new texas electoral map aimed keeping grip congress trump hail new texas electoral map aimed keeping grip congress trump hail new texas electoral map aimed keeping grip congress redistricting give party edge election redistricting give party edge election democrat mock jd vance cardboard charisma push unpopular budget bill opinion mayo pete buttigieg find seasoning happened ambition bay restoration guest commentary kilmar abrego garcia threatened deportation uganda larimer county restaurant inspection aug kilmar abrego garcia threatened deportation uganda kilmar abrego garcia threatened deportation uganda judge block trump cutting funding county denver sanctuary policy internet tax freedom act preempt new york imposition tax fbi target john boltons office trump smart guy unpatriotic guy inside facility training recruit take trump deportation goal inside facility training recruit take trump deportation goal inside facility training recruit take trump deportation goal inside facility training recruit take trump deportation goal rachel bitecofer warns bolton start trump rest inside facility training recruit take trump deportation goal inside facility training recruit take trump deportation goal inside facility training recruit take trump deportation goal china russia new strategic bomber inside facility training recruit take trump deportation goal inside facility training recruit take trump deportation goal zelenskyy security guarantee ukraine ready soon bill maher applauds gavin newsom mocking donald trump funny floridarun alligator alcatraz violates law aclu russia announces support venezuela defend sovereignty amid growing military tension united gianno caldwell mull senate bid chicagoans begging change crime woe trump threatens chicago next national guard invasion cnn analyst pinpoint weirdest part ghislaine maxwell simply bizarre doj interview cnn analyst pinpoint weirdest part ghislaine maxwell simply bizarre doj interview owl eye liberty memory epstein suicide trump clinton takeaway ghislaine maxwell transcript israel engineer famine gaza st century learned ghislaine maxwell doj interview texas gov abbott hell swiftly sign redistricting map lawmaker approve jeff bezos felt icky taken share amazon didnt feel good smart money strategy pro buy crypto market crash radioactive shrimp update walmart store brand brand recalled european postal service suspend shipment package tariff european postal service suspend shipment package tariff european postal service suspend shipment package tariff european postal service suspend shipment package tariff european postal service suspend shipment package tariff european postal service suspend shipment package tariff winning powerball ticket sold western new york sp hasnt yielded little since dotcom bubble investor motley fool ranked biggest financial stock pick best investment mezcal producer preserve traditional method demand liquor grows european postal service suspend shipment package tariff kpop demon hunter give netflix boxoffice curry join bank holiday sale bonanza epic deal event best offer id buy self driving taxi coming nyc waymo av testing permit mashable rosen leading law firm encourages fiserv investor secure counsel important rosen leading law firm encourages fiserv investor secure counsel important rosen leading law firm encourages fiserv investor secure counsel important rosen leading law firm encourages fiserv investor secure counsel important rosen leading law firm encourages fiserv investor secure counsel important deadline security class action fi cream sold walmarts across recalled due undeclared allergen gamestop purchase turned bitcoin jackpot cream sold walmarts across recalled due undeclared allergen fox business prediction lucid sale soar next year happens solar executive warn trump attack renewables lead power crunch spike electricity price pueblo county listing less money july median price prediction trilliondollar artificial intelligence ai stock strike megadeal wall street isnt ready cold wallet cashback utility presale pricing create upside case chainlink shiba inu struggle maintenance compliance burden viability hopi water treatment system ethereum trouble xrp breakout buyer turn blockdag earn referral reward acting executor lucrative job word national guard troop force multiplier homan little pepe crypto price prediction lilpepe good investment longterm holder aim invest invesco qqq etf million retirement audit federal spending moses lake school district blockchain stock worth watching august owner scale golden mile shopping center redevelopment rosen global investor counsel encourages easterly rocmuni high income municipal bond fund comerica bank lower stake alphabet goog trump tap airbnb cofounder st government design head lead web overhaul trump tap airbnb cofounder st government design head lead web overhaul fox business offgrid living next new real estate trend application rural mortgage skyrocket rosen global investor counsel encourages altimmune investor secure counsel rosen global investor counsel encourages altimmune investor secure counsel rosen global investor counsel encourages altimmune investor secure counsel epstein accuser virginia giuffre wrote memoir month death coming powell warning signal unemployment claim jump highest year cardano price outlook ada reach trumprelated defi platform world liberty financial debut wlfi token ethereum mainnet rosen global investor counsel encourages altimmune investor secure counsel important deadline security class action alt best meme coin presale stampede loading whitelist labubull watch moon without backtoschool deal tellos unlimited plan cell service per month month nexus gold cvenxs stock price whats next mason resource cvellg stock price mason resource cvellg trading happened national guard troop force multiplier homan freedom investment management purchase share procter gamble company pg ascent llc raise stock holding ameri</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>